<commit_message>
Update RQA header names for KPI_STRESS_SALES and DOWNGRADE
Both files now arrive with REPORT_DATE and VAL_AMT instead of the older
"REPORT DATE" and VALUES. Only colname_map changes; no tables added or
removed, and no other field touched.

reference.xlsx and tables_config.json were verified to be in sync --
regenerating the config from the spreadsheet reproduces the committed JSON
exactly. All 22 tables remain structurally coherent (every colname_map
still maps report_date/analytics/val_amt, and every kpi_analytics is still
a subset of its expected_analytics).

Note KPI_TRADING_PERF still uses "REPORT DATE"/"VALUES"; left as-is since
it is unclear whether RQA changed that extract too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ref/reference.xlsx
+++ b/ref/reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\appdata\mo-analytics\public\202606\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edsicage/Documents/claude-projects/mo-dq-checks/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492667FD-249C-4089-A920-8D339E02CD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D421EA2F-F099-A94D-8AD5-C1A21DEDC4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -95,9 +94,6 @@
     <t>template</t>
   </si>
   <si>
-    <t>{"REPORT DATE":"report_date", "MANDATE_ID":"mandate_id", "ANALYTICS":"analytics", "VALUES":"val_amt"}</t>
-  </si>
-  <si>
     <t>['port_stress_sales_ytd', 'port_stress_sales_3y']</t>
   </si>
   <si>
@@ -273,6 +269,9 @@
   </si>
   <si>
     <t>["report_date", "hr_mandate_id", "analytics"]</t>
+  </si>
+  <si>
+    <t>{"REPORT_DATE":"report_date", "MANDATE_ID":"mandate_id", "ANALYTICS":"analytics", "VAL_AMT":"val_amt"}</t>
   </si>
 </sst>
 </file>
@@ -669,21 +668,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultColWidth="22.54296875" defaultRowHeight="13" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="22.5" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.08984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.7265625" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="22.54296875" style="2"/>
+    <col min="5" max="5" width="22.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.6640625" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="22.5" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -712,10 +711,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="65" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="60" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -729,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -747,7 +746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="39" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -761,30 +760,30 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="52" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -793,10 +792,10 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>14</v>
@@ -805,467 +804,467 @@
         <v>15</v>
       </c>
       <c r="I4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="H7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="180" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="C11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="120" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="169" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="104" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" s="2" t="s">
+    <row r="14" spans="1:10" ht="195" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="195" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" s="2" t="s">
+    <row r="15" spans="1:10" ht="60" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="165" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="195" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="52" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="156" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="169" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I18" s="2" t="s">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I19" s="2" t="s">
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I20" s="2" t="s">
+    </row>
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="C21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>14</v>
@@ -1274,65 +1273,65 @@
         <v>15</v>
       </c>
       <c r="I21" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="120" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" ht="104" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="I22" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="39" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="J23" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>